<commit_message>
Merge Repository and SF10 menu items into one "Records & SF10"
The SF10 menu item opened the same Repository search page, so the sidebar
listed one page twice. SF10 is opened from each search result as before;
/permanent-record now redirects to the Repository. UAT steps for TC-043,
TC-045, TC-046, TC-048 and TC-062 follow the new name.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03-Testing/EduCheck_UAT_Test_Cases.xlsx
+++ b/03-Testing/EduCheck_UAT_Test_Cases.xlsx
@@ -3860,7 +3860,8 @@
       </c>
       <c r="I44" s="13" t="inlineStr">
         <is>
-          <t>1. Open Dashboard, Submission Review, Section Progress, Analytics, Digital Repository and SF10.</t>
+          <t>1. Open Dashboard, Submission Review, Section Progress, Analytics and Records &amp; SF10.
+2. In Records &amp; SF10, open a learner's Permanent Record (SF10).</t>
         </is>
       </c>
       <c r="J44" s="13" t="inlineStr">
@@ -3986,7 +3987,7 @@
       </c>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>1. Open Digital Repository.
+          <t>1. Open Records &amp; SF10.
 2. Search by LRN, then by name, then by grade level and school year.</t>
         </is>
       </c>
@@ -4050,7 +4051,7 @@
       </c>
       <c r="I47" s="13" t="inlineStr">
         <is>
-          <t>1. Open SF10 Permanent Records for the learner.
+          <t>1. Open Records &amp; SF10, search for the learner and click Permanent Record (SF10).
 2. Check the readiness report.
 3. Click Download and open the file in Excel.</t>
         </is>
@@ -4178,7 +4179,7 @@
       </c>
       <c r="I49" s="13" t="inlineStr">
         <is>
-          <t>1. Open the learner's SF10 page.
+          <t>1. Open Records &amp; SF10, search for the learner and click Permanent Record (SF10).
 2. Add a past school year with 4 quarter grades per subject and save.</t>
         </is>
       </c>
@@ -5072,7 +5073,7 @@
       </c>
       <c r="I63" s="13" t="inlineStr">
         <is>
-          <t>1. Open Dashboard, Consolidated Records, Analytics and Repository.
+          <t>1. Open Dashboard, Consolidated Records, Analytics and Records &amp; SF10.
 2. Time each page until its data appears.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
UAT: one file per subject, TC-068 for the subject check, TC-020/030 for partial departmentalization
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03-Testing/EduCheck_UAT_Test_Cases.xlsx
+++ b/03-Testing/EduCheck_UAT_Test_Cases.xlsx
@@ -1029,7 +1029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q68"/>
+  <dimension ref="A1:Q69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" style="25" min="1" max="1"/>
@@ -2395,7 +2395,7 @@
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>A section exists.</t>
+          <t>A section whose Adviser has no subject assignment.</t>
         </is>
       </c>
       <c r="I21" s="13" t="inlineStr">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="K21" s="13" t="inlineStr">
         <is>
-          <t>Self-Contained: the Adviser sees the upload page. Departmentalized: the Adviser's upload menu is hidden.</t>
+          <t>Self-Contained: the Adviser can upload every subject of the section. Departmentalized: the Adviser can upload only subjects assigned to them; with none, the upload menu is hidden. Switch the section back afterwards.</t>
         </is>
       </c>
       <c r="L21" s="16" t="n"/>
@@ -3025,28 +3025,29 @@
       </c>
       <c r="G31" s="13" t="inlineStr">
         <is>
-          <t>Self-Contained Adviser can upload</t>
+          <t>Adviser uploads their own assigned subject</t>
         </is>
       </c>
       <c r="H31" s="13" t="inlineStr">
         <is>
-          <t>Adviser of a Self-Contained section.</t>
+          <t>Rizal is Departmentalized and the Adviser is assigned at least one of its subjects.</t>
         </is>
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
           <t>1. Open Upload Files.
-2. Upload a record for a subject in the advisory section.</t>
+2. Check which subjects are offered for Rizal.
+3. Upload the file for one of the Adviser's own subjects.</t>
         </is>
       </c>
       <c r="J31" s="13" t="inlineStr">
         <is>
-          <t>adviser.grade6a, Rizal, UAT-files/TC-022_valid-ecr-rizal.xlsx</t>
+          <t>adviser.grade6a, Rizal, the matching file from UAT-files/per-subject/</t>
         </is>
       </c>
       <c r="K31" s="13" t="inlineStr">
         <is>
-          <t>Upload succeeds as for a Subject Teacher.</t>
+          <t>Only the Adviser's own subjects are offered. The upload succeeds as for a Subject Teacher.</t>
         </is>
       </c>
       <c r="L31" s="16" t="n"/>
@@ -5409,6 +5410,71 @@
       <c r="O68" s="18" t="n"/>
       <c r="P68" s="17" t="n"/>
       <c r="Q68" s="16" t="n"/>
+    </row>
+    <row r="69" ht="30" customHeight="1" s="25">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>TC-068</t>
+        </is>
+      </c>
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>Upload</t>
+        </is>
+      </c>
+      <c r="C69" s="15" t="inlineStr">
+        <is>
+          <t>Subject Teacher</t>
+        </is>
+      </c>
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E69" s="13" t="inlineStr">
+        <is>
+          <t>Functional suitability</t>
+        </is>
+      </c>
+      <c r="F69" s="13" t="inlineStr">
+        <is>
+          <t>EPIC-02, D-08</t>
+        </is>
+      </c>
+      <c r="G69" s="13" t="inlineStr">
+        <is>
+          <t>A file for another subject is refused</t>
+        </is>
+      </c>
+      <c r="H69" s="13" t="inlineStr">
+        <is>
+          <t>Teacher is assigned to Mathematics for Rizal. No Rizal learner is Approved.</t>
+        </is>
+      </c>
+      <c r="I69" s="13" t="inlineStr">
+        <is>
+          <t>1. Open Upload e-Class Record.
+2. Select Mathematics and Rizal.
+3. Upload the English file.</t>
+        </is>
+      </c>
+      <c r="J69" s="13" t="inlineStr">
+        <is>
+          <t>UAT-files/per-subject/ecr-rizal-English.xlsx</t>
+        </is>
+      </c>
+      <c r="K69" s="13" t="inlineStr">
+        <is>
+          <t>The upload is refused: the file is the e-Class Record for English but Mathematics was selected. Nothing is saved.</t>
+        </is>
+      </c>
+      <c r="L69" s="16" t="n"/>
+      <c r="M69" s="17" t="n"/>
+      <c r="N69" s="16" t="n"/>
+      <c r="O69" s="18" t="n"/>
+      <c r="P69" s="17" t="n"/>
+      <c r="Q69" s="16" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q68"/>
@@ -5427,10 +5493,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="M2:M68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Status" error="Choose Pass, Fail, Blocked or Not Run." type="list">
+    <dataValidation sqref="M2:M69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Status" error="Choose Pass, Fail, Blocked or Not Run." type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O68" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Enter a date (YYYY-MM-DD)." type="date" operator="greaterThan">
+    <dataValidation sqref="O2:O69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Enter a date (YYYY-MM-DD)." type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -5466,6 +5532,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -5480,7 +5547,7 @@
         </is>
       </c>
       <c r="B5" s="20">
-        <f>COUNTA('Test Cases'!$A$2:$A$68)</f>
+        <f>COUNTA('Test Cases'!$A$2:$A$69)</f>
         <v/>
       </c>
     </row>
@@ -5491,7 +5558,7 @@
         </is>
       </c>
       <c r="B6" s="20">
-        <f>COUNTIF('Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIF('Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -5502,7 +5569,7 @@
         </is>
       </c>
       <c r="B7" s="20">
-        <f>COUNTIF('Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIF('Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -5513,7 +5580,7 @@
         </is>
       </c>
       <c r="B8" s="20">
-        <f>COUNTIF('Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIF('Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -5561,6 +5628,8 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="19" t="inlineStr">
         <is>
@@ -5612,19 +5681,19 @@
         </is>
       </c>
       <c r="B17" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A17)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A17)</f>
         <v/>
       </c>
       <c r="C17" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A17,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A17,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A17,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A17,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A17,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A17,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F17" s="20">
@@ -5643,19 +5712,19 @@
         </is>
       </c>
       <c r="B18" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A18)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A18)</f>
         <v/>
       </c>
       <c r="C18" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A18,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A18,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A18,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A18,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A18,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A18,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F18" s="20">
@@ -5674,19 +5743,19 @@
         </is>
       </c>
       <c r="B19" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A19)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A19)</f>
         <v/>
       </c>
       <c r="C19" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A19,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A19,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A19,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A19,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A19,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A19,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F19" s="20">
@@ -5705,19 +5774,19 @@
         </is>
       </c>
       <c r="B20" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A20)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A20)</f>
         <v/>
       </c>
       <c r="C20" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A20,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A20,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A20,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A20,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A20,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A20,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F20" s="20">
@@ -5736,19 +5805,19 @@
         </is>
       </c>
       <c r="B21" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A21)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A21)</f>
         <v/>
       </c>
       <c r="C21" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A21,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A21,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A21,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A21,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A21,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A21,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F21" s="20">
@@ -5767,19 +5836,19 @@
         </is>
       </c>
       <c r="B22" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A22)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A22)</f>
         <v/>
       </c>
       <c r="C22" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A22,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A22,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A22,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A22,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A22,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A22,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F22" s="20">
@@ -5798,19 +5867,19 @@
         </is>
       </c>
       <c r="B23" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A23)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A23)</f>
         <v/>
       </c>
       <c r="C23" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A23,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A23,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D23" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A23,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A23,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E23" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A23,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A23,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F23" s="20">
@@ -5829,19 +5898,19 @@
         </is>
       </c>
       <c r="B24" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A24)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A24)</f>
         <v/>
       </c>
       <c r="C24" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A24,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A24,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D24" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A24,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A24,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E24" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A24,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A24,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F24" s="20">
@@ -5860,19 +5929,19 @@
         </is>
       </c>
       <c r="B25" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A25)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A25)</f>
         <v/>
       </c>
       <c r="C25" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A25,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A25,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D25" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A25,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A25,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E25" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A25,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A25,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F25" s="20">
@@ -5891,19 +5960,19 @@
         </is>
       </c>
       <c r="B26" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A26)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A26)</f>
         <v/>
       </c>
       <c r="C26" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A26,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A26,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A26,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A26,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A26,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A26,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F26" s="20">
@@ -5922,19 +5991,19 @@
         </is>
       </c>
       <c r="B27" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A27)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A27)</f>
         <v/>
       </c>
       <c r="C27" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A27,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A27,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A27,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A27,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A27,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A27,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F27" s="20">
@@ -5953,19 +6022,19 @@
         </is>
       </c>
       <c r="B28" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A28)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A28)</f>
         <v/>
       </c>
       <c r="C28" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A28,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A28,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A28,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A28,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A28,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A28,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F28" s="20">
@@ -5984,19 +6053,19 @@
         </is>
       </c>
       <c r="B29" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A29)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A29)</f>
         <v/>
       </c>
       <c r="C29" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A29,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A29,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D29" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A29,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A29,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E29" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A29,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A29,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F29" s="20">
@@ -6015,19 +6084,19 @@
         </is>
       </c>
       <c r="B30" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A30)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A30)</f>
         <v/>
       </c>
       <c r="C30" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A30,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A30,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D30" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A30,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A30,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E30" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A30,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A30,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F30" s="20">
@@ -6046,19 +6115,19 @@
         </is>
       </c>
       <c r="B31" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A31)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A31)</f>
         <v/>
       </c>
       <c r="C31" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A31,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A31,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D31" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A31,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A31,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E31" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A31,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A31,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F31" s="20">
@@ -6077,19 +6146,19 @@
         </is>
       </c>
       <c r="B32" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A32)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A32)</f>
         <v/>
       </c>
       <c r="C32" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A32,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A32,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D32" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A32,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A32,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E32" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A32,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A32,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F32" s="20">
@@ -6108,19 +6177,19 @@
         </is>
       </c>
       <c r="B33" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A33)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A33)</f>
         <v/>
       </c>
       <c r="C33" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A33,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A33,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D33" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A33,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A33,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E33" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A33,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A33,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F33" s="20">
@@ -6139,19 +6208,19 @@
         </is>
       </c>
       <c r="B34" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A34)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A34)</f>
         <v/>
       </c>
       <c r="C34" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A34,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A34,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D34" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A34,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A34,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E34" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A34,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A34,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F34" s="20">
@@ -6170,19 +6239,19 @@
         </is>
       </c>
       <c r="B35" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A35)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A35)</f>
         <v/>
       </c>
       <c r="C35" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A35,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A35,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D35" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A35,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A35,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E35" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A35,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A35,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F35" s="20">
@@ -6201,19 +6270,19 @@
         </is>
       </c>
       <c r="B36" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A36)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A36)</f>
         <v/>
       </c>
       <c r="C36" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A36,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A36,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D36" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A36,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A36,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E36" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A36,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A36,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F36" s="20">
@@ -6232,19 +6301,19 @@
         </is>
       </c>
       <c r="B37" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A37)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A37)</f>
         <v/>
       </c>
       <c r="C37" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A37,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A37,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D37" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A37,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A37,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E37" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A37,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A37,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F37" s="20">
@@ -6263,19 +6332,19 @@
         </is>
       </c>
       <c r="B38" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$68,A38)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$69,A38)</f>
         <v/>
       </c>
       <c r="C38" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A38,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A38,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D38" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A38,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A38,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E38" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$68,A38,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A38,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F38" s="20">
@@ -6287,6 +6356,8 @@
         <v/>
       </c>
     </row>
+    <row r="39"/>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="19" t="inlineStr">
         <is>
@@ -6338,19 +6409,19 @@
         </is>
       </c>
       <c r="B43" s="20">
-        <f>COUNTIF('Test Cases'!$E$2:$E$68,A43)</f>
+        <f>COUNTIF('Test Cases'!$E$2:$E$69,A43)</f>
         <v/>
       </c>
       <c r="C43" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A43,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A43,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D43" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A43,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A43,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E43" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A43,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A43,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F43" s="20">
@@ -6369,19 +6440,19 @@
         </is>
       </c>
       <c r="B44" s="20">
-        <f>COUNTIF('Test Cases'!$E$2:$E$68,A44)</f>
+        <f>COUNTIF('Test Cases'!$E$2:$E$69,A44)</f>
         <v/>
       </c>
       <c r="C44" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A44,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A44,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D44" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A44,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A44,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E44" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A44,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A44,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F44" s="20">
@@ -6400,19 +6471,19 @@
         </is>
       </c>
       <c r="B45" s="20">
-        <f>COUNTIF('Test Cases'!$E$2:$E$68,A45)</f>
+        <f>COUNTIF('Test Cases'!$E$2:$E$69,A45)</f>
         <v/>
       </c>
       <c r="C45" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A45,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A45,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D45" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A45,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A45,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E45" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A45,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A45,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F45" s="20">
@@ -6431,19 +6502,19 @@
         </is>
       </c>
       <c r="B46" s="20">
-        <f>COUNTIF('Test Cases'!$E$2:$E$68,A46)</f>
+        <f>COUNTIF('Test Cases'!$E$2:$E$69,A46)</f>
         <v/>
       </c>
       <c r="C46" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A46,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A46,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D46" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A46,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A46,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E46" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A46,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A46,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F46" s="20">
@@ -6462,19 +6533,19 @@
         </is>
       </c>
       <c r="B47" s="20">
-        <f>COUNTIF('Test Cases'!$E$2:$E$68,A47)</f>
+        <f>COUNTIF('Test Cases'!$E$2:$E$69,A47)</f>
         <v/>
       </c>
       <c r="C47" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A47,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A47,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D47" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A47,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A47,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E47" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A47,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A47,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F47" s="20">
@@ -6493,19 +6564,19 @@
         </is>
       </c>
       <c r="B48" s="20">
-        <f>COUNTIF('Test Cases'!$E$2:$E$68,A48)</f>
+        <f>COUNTIF('Test Cases'!$E$2:$E$69,A48)</f>
         <v/>
       </c>
       <c r="C48" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A48,'Test Cases'!$M$2:$M$68,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A48,'Test Cases'!$M$2:$M$69,"Pass")</f>
         <v/>
       </c>
       <c r="D48" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A48,'Test Cases'!$M$2:$M$68,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A48,'Test Cases'!$M$2:$M$69,"Fail")</f>
         <v/>
       </c>
       <c r="E48" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$68,A48,'Test Cases'!$M$2:$M$68,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A48,'Test Cases'!$M$2:$M$69,"Blocked")</f>
         <v/>
       </c>
       <c r="F48" s="20">

</xml_diff>

<commit_message>
Assign several subjects to a teacher in one save
Add Assignment now shows a checklist of the section's own grade-level
subjects plus the Class Adviser slot, so an Adviser or Subject Teacher
with several subjects is set up in one save instead of one form per
subject. Slots already held show who holds them; the Class Adviser box
needs an Adviser account.

New POST /api/assignments/batch applies the existing rules to every item
and saves all-or-nothing in one transaction; the single-assignment
endpoint is unchanged. Tests BAT-01 to BAT-07; UAT TC-017 to TC-019
updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03-Testing/EduCheck_UAT_Test_Cases.xlsx
+++ b/03-Testing/EduCheck_UAT_Test_Cases.xlsx
@@ -2199,28 +2199,29 @@
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>Assign a Subject Teacher to a subject and section</t>
+          <t>Assign a teacher to several subjects of a section in one save</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>A section, a Subject Teacher and the subject exist.</t>
+          <t>A section, a teacher, and subjects of the section's grade level not yet assigned.</t>
         </is>
       </c>
       <c r="I18" s="13" t="inlineStr">
         <is>
-          <t>1. Open Section &amp; Teacher Assignments.
-2. Assign the teacher to a subject for a section of the same grade level.</t>
+          <t>1. Open Section &amp; Teacher Assignments and click Add Assignment.
+2. Choose the teacher, section and school year.
+3. Tick two or more subjects and save.</t>
         </is>
       </c>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>e.g. Grade 6 English to Rizal</t>
+          <t>e.g. Grade 6 English and Science to Rizal</t>
         </is>
       </c>
       <c r="K18" s="13" t="inlineStr">
         <is>
-          <t>The assignment is saved. The teacher now sees that subject and section on the upload page.</t>
+          <t>One save creates every ticked assignment, each listed separately. Subjects already held by another teacher show who holds them and cannot be ticked. The teacher now sees those subjects for that section on the upload page.</t>
         </is>
       </c>
       <c r="L18" s="16" t="n"/>
@@ -2263,7 +2264,7 @@
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>Grade-level mismatch is rejected</t>
+          <t>Only the section's own grade-level subjects are offered</t>
         </is>
       </c>
       <c r="H19" s="13" t="inlineStr">
@@ -2273,17 +2274,18 @@
       </c>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>1. Try to assign a Grade 3 subject to a Grade 6 section.</t>
+          <t>1. Open Add Assignment and choose a Grade 6 section.
+2. Look at the subject checklist.</t>
         </is>
       </c>
       <c r="J19" s="13" t="inlineStr">
         <is>
-          <t>Grade 3 subject, Rizal (Grade 6)</t>
+          <t>Rizal (Grade 6)</t>
         </is>
       </c>
       <c r="K19" s="13" t="inlineStr">
         <is>
-          <t>The assignment is refused with a message that the grade levels do not match.</t>
+          <t>Only Grade 6 subjects are listed, so a subject from another grade level cannot be chosen.</t>
         </is>
       </c>
       <c r="L19" s="16" t="n"/>
@@ -2336,8 +2338,9 @@
       </c>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>1. Choose a teacher with a Subject Teacher account.
-2. Leave Subject blank (Class Adviser) and save.</t>
+          <t>1. Open Add Assignment.
+2. Choose a teacher with a Subject Teacher account and a section without a Class Adviser.
+3. Look at the Class Adviser box.</t>
         </is>
       </c>
       <c r="J20" s="13" t="inlineStr">
@@ -2347,7 +2350,7 @@
       </c>
       <c r="K20" s="13" t="inlineStr">
         <is>
-          <t>The assignment is refused with a message that only an Adviser account can be Class Adviser. The section's Adviser slot stays free.</t>
+          <t>The Class Adviser box cannot be ticked and says it needs an Adviser account. The section's Adviser slot stays free.</t>
         </is>
       </c>
       <c r="L20" s="16" t="n"/>
@@ -5532,7 +5535,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -5628,8 +5630,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="19" t="inlineStr">
         <is>
@@ -6356,8 +6356,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Print 3-term years on the SF10 and import earlier years from an SF10 file
On the capstone adviser's direction, a 3-term year keeps the official SF10-ES form and uses three of its block's four rating columns, relabelled T1-T3, with the fourth left blank; terms are printed as recorded, never converted. 4-quarter years are unchanged.

Earlier years can now also be imported from the learner's existing SF10-ES file: the server reads every filled Grade 1-6 block (including the Back sheet's inline headers), refuses another learner's file, and returns a preview; the page saves only the ticked years through the normal historical entry, so validation and the audit log are the same as typed years.

Tests: SF-07/10/11 updated, SF-14 round trip, SF-15 import then print, SF-16 refusals. Known Limitations D-05 updated, D-09 added; UAT TC-047 updated, TC-069 to TC-071 added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03-Testing/EduCheck_UAT_Test_Cases.xlsx
+++ b/03-Testing/EduCheck_UAT_Test_Cases.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11328" yWindow="0" windowWidth="11712" windowHeight="12240" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Test Cases" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Defect Log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defect Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Cases'!$A$1:$Q$68</definedName>
@@ -1029,7 +1029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q69"/>
+  <dimension ref="A1:Q72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" style="25" min="1" max="1"/>
@@ -4105,7 +4105,7 @@
       </c>
       <c r="F48" s="13" t="inlineStr">
         <is>
-          <t>D-05</t>
+          <t>US-005</t>
         </is>
       </c>
       <c r="G48" s="13" t="inlineStr">
@@ -4115,7 +4115,7 @@
       </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
-          <t>Learner has only a 3-term year.</t>
+          <t>Learner's only year is a 2025-2026 EduCheck record that is not yet approved.</t>
         </is>
       </c>
       <c r="I48" s="13" t="inlineStr">
@@ -5478,6 +5478,201 @@
       <c r="O69" s="18" t="n"/>
       <c r="P69" s="17" t="n"/>
       <c r="Q69" s="16" t="n"/>
+    </row>
+    <row r="70" ht="30" customHeight="1" s="25">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>TC-069</t>
+        </is>
+      </c>
+      <c r="B70" s="13" t="inlineStr">
+        <is>
+          <t>SF10</t>
+        </is>
+      </c>
+      <c r="C70" s="15" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E70" s="13" t="inlineStr">
+        <is>
+          <t>Functional suitability</t>
+        </is>
+      </c>
+      <c r="F70" s="13" t="inlineStr">
+        <is>
+          <t>D-05, US-005</t>
+        </is>
+      </c>
+      <c r="G70" s="13" t="inlineStr">
+        <is>
+          <t>A 3-term year prints as Terms 1-3</t>
+        </is>
+      </c>
+      <c r="H70" s="13" t="inlineStr">
+        <is>
+          <t>A Rizal learner's 2025-2026 record has been approved (e.g. after TC-039).</t>
+        </is>
+      </c>
+      <c r="I70" s="13" t="inlineStr">
+        <is>
+          <t>1. Open Records &amp; SF10 and open that learner's Permanent Record (SF10).
+2. Check the Grade 6 card.
+3. Click Generate SF10 and open the file in Excel (Back sheet, Grade 6).</t>
+        </is>
+      </c>
+      <c r="J70" s="13" t="inlineStr">
+        <is>
+          <t>LRN of the approved learner</t>
+        </is>
+      </c>
+      <c r="K70" s="13" t="inlineStr">
+        <is>
+          <t>The Grade 6 card says it was graded in 3 terms. In the file, the Grade 6 block is headed "Term Rating" with columns T1, T2, T3 and –; each learning area shows its three term grades, final rating and remarks; the fourth column is empty; the school details are Atimonan Central School Annex.</t>
+        </is>
+      </c>
+      <c r="L70" s="16" t="n"/>
+      <c r="M70" s="17" t="n"/>
+      <c r="N70" s="16" t="n"/>
+      <c r="O70" s="18" t="n"/>
+      <c r="P70" s="17" t="n"/>
+      <c r="Q70" s="16" t="n"/>
+    </row>
+    <row r="71" ht="30" customHeight="1" s="25">
+      <c r="A71" s="14" t="inlineStr">
+        <is>
+          <t>TC-070</t>
+        </is>
+      </c>
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>SF10</t>
+        </is>
+      </c>
+      <c r="C71" s="15" t="inlineStr">
+        <is>
+          <t>Adviser</t>
+        </is>
+      </c>
+      <c r="D71" s="15" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E71" s="13" t="inlineStr">
+        <is>
+          <t>Functional suitability</t>
+        </is>
+      </c>
+      <c r="F71" s="13" t="inlineStr">
+        <is>
+          <t>US-014</t>
+        </is>
+      </c>
+      <c r="G71" s="13" t="inlineStr">
+        <is>
+          <t>Import earlier years from an existing SF10 file</t>
+        </is>
+      </c>
+      <c r="H71" s="13" t="inlineStr">
+        <is>
+          <t>Logged in as the Rizal Adviser. Learner 100000000001 has Grade 4 and Grade 5 records.</t>
+        </is>
+      </c>
+      <c r="I71" s="13" t="inlineStr">
+        <is>
+          <t>1. Open the Permanent Record of 100000000001 and click Generate SF10 to save a copy.
+2. Delete the Grade 5 year.
+3. Click Import from SF10 and choose the saved file.
+4. Check the preview, keep only Grade 5 ticked and click Import.</t>
+        </is>
+      </c>
+      <c r="J71" s="13" t="inlineStr">
+        <is>
+          <t>LRN 100000000001; the SF10 file from step 1</t>
+        </is>
+      </c>
+      <c r="K71" s="13" t="inlineStr">
+        <is>
+          <t>The preview lists Grade 4 and Grade 5 with school year, grading, number of learning areas and general average, and nothing is saved until Import is clicked. Grade 5 is restored with the same grades, appears in the readiness report and in a newly generated SF10, and the save is in the Audit Log.</t>
+        </is>
+      </c>
+      <c r="L71" s="16" t="n"/>
+      <c r="M71" s="17" t="n"/>
+      <c r="N71" s="16" t="n"/>
+      <c r="O71" s="18" t="n"/>
+      <c r="P71" s="17" t="n"/>
+      <c r="Q71" s="16" t="n"/>
+    </row>
+    <row r="72" ht="30" customHeight="1" s="25">
+      <c r="A72" s="14" t="inlineStr">
+        <is>
+          <t>TC-071</t>
+        </is>
+      </c>
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>SF10</t>
+        </is>
+      </c>
+      <c r="C72" s="15" t="inlineStr">
+        <is>
+          <t>Adviser</t>
+        </is>
+      </c>
+      <c r="D72" s="15" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="E72" s="13" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="F72" s="13" t="inlineStr">
+        <is>
+          <t>US-014</t>
+        </is>
+      </c>
+      <c r="G72" s="13" t="inlineStr">
+        <is>
+          <t>Import refuses another learner's SF10</t>
+        </is>
+      </c>
+      <c r="H72" s="13" t="inlineStr">
+        <is>
+          <t>Logged in as the Rizal Adviser. The SF10 file of 100000000001 from TC-070.</t>
+        </is>
+      </c>
+      <c r="I72" s="13" t="inlineStr">
+        <is>
+          <t>1. Open the Permanent Record of another Rizal learner.
+2. Click Import from SF10 and choose 100000000001's file.</t>
+        </is>
+      </c>
+      <c r="J72" s="13" t="inlineStr">
+        <is>
+          <t>e.g. LRN 100000000004</t>
+        </is>
+      </c>
+      <c r="K72" s="13" t="inlineStr">
+        <is>
+          <t>The import is refused with a message that the SF10 belongs to LRN 100000000001. Nothing is saved.</t>
+        </is>
+      </c>
+      <c r="L72" s="16" t="n"/>
+      <c r="M72" s="17" t="n"/>
+      <c r="N72" s="16" t="n"/>
+      <c r="O72" s="18" t="n"/>
+      <c r="P72" s="17" t="n"/>
+      <c r="Q72" s="16" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:Q68"/>
@@ -5496,10 +5691,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="M2:M69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Status" error="Choose Pass, Fail, Blocked or Not Run." type="list">
+    <dataValidation sqref="M2:M72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Status" error="Choose Pass, Fail, Blocked or Not Run." type="list">
       <formula1>"Pass,Fail,Blocked,Not Run"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Enter a date (YYYY-MM-DD)." type="date" operator="greaterThan">
+    <dataValidation sqref="O2:O72" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Enter a date (YYYY-MM-DD)." type="date" operator="greaterThan">
       <formula1>DATE(2026,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -5535,6 +5730,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -5549,7 +5745,7 @@
         </is>
       </c>
       <c r="B5" s="20">
-        <f>COUNTA('Test Cases'!$A$2:$A$69)</f>
+        <f>COUNTA('Test Cases'!$A$2:$A$72)</f>
         <v/>
       </c>
     </row>
@@ -5560,7 +5756,7 @@
         </is>
       </c>
       <c r="B6" s="20">
-        <f>COUNTIF('Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIF('Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -5571,7 +5767,7 @@
         </is>
       </c>
       <c r="B7" s="20">
-        <f>COUNTIF('Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIF('Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -5582,7 +5778,7 @@
         </is>
       </c>
       <c r="B8" s="20">
-        <f>COUNTIF('Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIF('Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -5630,6 +5826,8 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="19" t="inlineStr">
         <is>
@@ -5681,19 +5879,19 @@
         </is>
       </c>
       <c r="B17" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A17)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A17)</f>
         <v/>
       </c>
       <c r="C17" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A17,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A17,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D17" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A17,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A17,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E17" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A17,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A17,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F17" s="20">
@@ -5712,19 +5910,19 @@
         </is>
       </c>
       <c r="B18" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A18)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A18)</f>
         <v/>
       </c>
       <c r="C18" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A18,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A18,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D18" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A18,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A18,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E18" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A18,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A18,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F18" s="20">
@@ -5743,19 +5941,19 @@
         </is>
       </c>
       <c r="B19" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A19)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A19)</f>
         <v/>
       </c>
       <c r="C19" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A19,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A19,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D19" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A19,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A19,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E19" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A19,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A19,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F19" s="20">
@@ -5774,19 +5972,19 @@
         </is>
       </c>
       <c r="B20" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A20)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A20)</f>
         <v/>
       </c>
       <c r="C20" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A20,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A20,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D20" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A20,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A20,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E20" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A20,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A20,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F20" s="20">
@@ -5805,19 +6003,19 @@
         </is>
       </c>
       <c r="B21" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A21)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A21)</f>
         <v/>
       </c>
       <c r="C21" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A21,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A21,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D21" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A21,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A21,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E21" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A21,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A21,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F21" s="20">
@@ -5836,19 +6034,19 @@
         </is>
       </c>
       <c r="B22" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A22)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A22)</f>
         <v/>
       </c>
       <c r="C22" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A22,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A22,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A22,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A22,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A22,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A22,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F22" s="20">
@@ -5867,19 +6065,19 @@
         </is>
       </c>
       <c r="B23" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A23)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A23)</f>
         <v/>
       </c>
       <c r="C23" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A23,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A23,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D23" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A23,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A23,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E23" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A23,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A23,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F23" s="20">
@@ -5898,19 +6096,19 @@
         </is>
       </c>
       <c r="B24" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A24)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A24)</f>
         <v/>
       </c>
       <c r="C24" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A24,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A24,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D24" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A24,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A24,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E24" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A24,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A24,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F24" s="20">
@@ -5929,19 +6127,19 @@
         </is>
       </c>
       <c r="B25" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A25)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A25)</f>
         <v/>
       </c>
       <c r="C25" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A25,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A25,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D25" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A25,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A25,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E25" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A25,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A25,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F25" s="20">
@@ -5960,19 +6158,19 @@
         </is>
       </c>
       <c r="B26" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A26)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A26)</f>
         <v/>
       </c>
       <c r="C26" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A26,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A26,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D26" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A26,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A26,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E26" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A26,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A26,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F26" s="20">
@@ -5991,19 +6189,19 @@
         </is>
       </c>
       <c r="B27" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A27)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A27)</f>
         <v/>
       </c>
       <c r="C27" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A27,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A27,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D27" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A27,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A27,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E27" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A27,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A27,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F27" s="20">
@@ -6022,19 +6220,19 @@
         </is>
       </c>
       <c r="B28" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A28)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A28)</f>
         <v/>
       </c>
       <c r="C28" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A28,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A28,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D28" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A28,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A28,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E28" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A28,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A28,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F28" s="20">
@@ -6053,19 +6251,19 @@
         </is>
       </c>
       <c r="B29" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A29)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A29)</f>
         <v/>
       </c>
       <c r="C29" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A29,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A29,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D29" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A29,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A29,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E29" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A29,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A29,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F29" s="20">
@@ -6084,19 +6282,19 @@
         </is>
       </c>
       <c r="B30" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A30)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A30)</f>
         <v/>
       </c>
       <c r="C30" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A30,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A30,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D30" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A30,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A30,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E30" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A30,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A30,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F30" s="20">
@@ -6115,19 +6313,19 @@
         </is>
       </c>
       <c r="B31" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A31)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A31)</f>
         <v/>
       </c>
       <c r="C31" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A31,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A31,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D31" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A31,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A31,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E31" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A31,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A31,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F31" s="20">
@@ -6146,19 +6344,19 @@
         </is>
       </c>
       <c r="B32" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A32)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A32)</f>
         <v/>
       </c>
       <c r="C32" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A32,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A32,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D32" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A32,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A32,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E32" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A32,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A32,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F32" s="20">
@@ -6177,19 +6375,19 @@
         </is>
       </c>
       <c r="B33" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A33)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A33)</f>
         <v/>
       </c>
       <c r="C33" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A33,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A33,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D33" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A33,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A33,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E33" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A33,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A33,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F33" s="20">
@@ -6208,19 +6406,19 @@
         </is>
       </c>
       <c r="B34" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A34)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A34)</f>
         <v/>
       </c>
       <c r="C34" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A34,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A34,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D34" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A34,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A34,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E34" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A34,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A34,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F34" s="20">
@@ -6239,19 +6437,19 @@
         </is>
       </c>
       <c r="B35" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A35)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A35)</f>
         <v/>
       </c>
       <c r="C35" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A35,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A35,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D35" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A35,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A35,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E35" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A35,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A35,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F35" s="20">
@@ -6270,19 +6468,19 @@
         </is>
       </c>
       <c r="B36" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A36)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A36)</f>
         <v/>
       </c>
       <c r="C36" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A36,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A36,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D36" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A36,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A36,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E36" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A36,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A36,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F36" s="20">
@@ -6301,19 +6499,19 @@
         </is>
       </c>
       <c r="B37" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A37)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A37)</f>
         <v/>
       </c>
       <c r="C37" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A37,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A37,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D37" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A37,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A37,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E37" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A37,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A37,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F37" s="20">
@@ -6332,19 +6530,19 @@
         </is>
       </c>
       <c r="B38" s="20">
-        <f>COUNTIF('Test Cases'!$B$2:$B$69,A38)</f>
+        <f>COUNTIF('Test Cases'!$B$2:$B$72,A38)</f>
         <v/>
       </c>
       <c r="C38" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A38,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A38,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D38" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A38,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A38,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E38" s="20">
-        <f>COUNTIFS('Test Cases'!$B$2:$B$69,A38,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$B$2:$B$72,A38,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F38" s="20">
@@ -6356,6 +6554,8 @@
         <v/>
       </c>
     </row>
+    <row r="39"/>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="19" t="inlineStr">
         <is>
@@ -6407,19 +6607,19 @@
         </is>
       </c>
       <c r="B43" s="20">
-        <f>COUNTIF('Test Cases'!$E$2:$E$69,A43)</f>
+        <f>COUNTIF('Test Cases'!$E$2:$E$72,A43)</f>
         <v/>
       </c>
       <c r="C43" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A43,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A43,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D43" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A43,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A43,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E43" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A43,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A43,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F43" s="20">
@@ -6438,19 +6638,19 @@
         </is>
       </c>
       <c r="B44" s="20">
-        <f>COUNTIF('Test Cases'!$E$2:$E$69,A44)</f>
+        <f>COUNTIF('Test Cases'!$E$2:$E$72,A44)</f>
         <v/>
       </c>
       <c r="C44" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A44,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A44,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D44" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A44,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A44,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E44" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A44,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A44,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F44" s="20">
@@ -6469,19 +6669,19 @@
         </is>
       </c>
       <c r="B45" s="20">
-        <f>COUNTIF('Test Cases'!$E$2:$E$69,A45)</f>
+        <f>COUNTIF('Test Cases'!$E$2:$E$72,A45)</f>
         <v/>
       </c>
       <c r="C45" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A45,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A45,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D45" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A45,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A45,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E45" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A45,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A45,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F45" s="20">
@@ -6500,19 +6700,19 @@
         </is>
       </c>
       <c r="B46" s="20">
-        <f>COUNTIF('Test Cases'!$E$2:$E$69,A46)</f>
+        <f>COUNTIF('Test Cases'!$E$2:$E$72,A46)</f>
         <v/>
       </c>
       <c r="C46" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A46,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A46,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D46" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A46,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A46,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E46" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A46,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A46,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F46" s="20">
@@ -6531,19 +6731,19 @@
         </is>
       </c>
       <c r="B47" s="20">
-        <f>COUNTIF('Test Cases'!$E$2:$E$69,A47)</f>
+        <f>COUNTIF('Test Cases'!$E$2:$E$72,A47)</f>
         <v/>
       </c>
       <c r="C47" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A47,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A47,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D47" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A47,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A47,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E47" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A47,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A47,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F47" s="20">
@@ -6562,19 +6762,19 @@
         </is>
       </c>
       <c r="B48" s="20">
-        <f>COUNTIF('Test Cases'!$E$2:$E$69,A48)</f>
+        <f>COUNTIF('Test Cases'!$E$2:$E$72,A48)</f>
         <v/>
       </c>
       <c r="C48" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A48,'Test Cases'!$M$2:$M$69,"Pass")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A48,'Test Cases'!$M$2:$M$72,"Pass")</f>
         <v/>
       </c>
       <c r="D48" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A48,'Test Cases'!$M$2:$M$69,"Fail")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A48,'Test Cases'!$M$2:$M$72,"Fail")</f>
         <v/>
       </c>
       <c r="E48" s="20">
-        <f>COUNTIFS('Test Cases'!$E$2:$E$69,A48,'Test Cases'!$M$2:$M$69,"Blocked")</f>
+        <f>COUNTIFS('Test Cases'!$E$2:$E$72,A48,'Test Cases'!$M$2:$M$72,"Blocked")</f>
         <v/>
       </c>
       <c r="F48" s="20">

</xml_diff>

<commit_message>
Add the UAT Day Kit; keep two learners incomplete for TC-036
The Day Kit has the dry-run and morning checklists, the 10-minute orientation script, the session flow and a run sheet per role in a dependency-safe order (approve 004 for the SF10 check and 006 for the amendment; TC-047 uses an unapproved learner).

The TLE file now leaves out LRN 100000000099 and 100000000100 again so TC-036 has incomplete learners. Workbook: TC-047 data and the Instructions sheet updated for the Departmentalized setup and fictitious names.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03-Testing/EduCheck_UAT_Test_Cases.xlsx
+++ b/03-Testing/EduCheck_UAT_Test_Cases.xlsx
@@ -908,7 +908,7 @@
       <c r="C33" s="6" t="n"/>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>Adviser of Rizal (Grade 6, Self-Contained).</t>
+          <t>Maria Teresa Santos (fictitious name). Class Adviser of Rizal (Grade 6, Departmentalized); teaches English, ESP, Filipino and Science.</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       <c r="C34" s="6" t="n"/>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>Uploads e-class records.</t>
+          <t>Jose Miguel Reyes (fictitious name). Teaches Araling Panlipunan, MAPEH, Mathematics and TLE in Rizal.</t>
         </is>
       </c>
     </row>
@@ -966,7 +966,7 @@
       </c>
       <c r="B38" s="24" t="inlineStr">
         <is>
-          <t>Rizal (Grade 6, Self-Contained, 100 learners). Mabini (Grade 3, Departmentalized, 5 learners LRN 300000000001-005, no Class Adviser). School year 2025-2026. Pending Approval at start: LRN 100000000004-015. Incomplete (no TLE grade): LRN 100000000099 and 100000000100. No Approved records at start.</t>
+          <t>Rizal (Grade 6, Departmentalized, 100 learners). Mabini (Grade 3, Self-Contained, 5 learners LRN 300000000001-005, no Class Adviser). School year 2025-2026. Pending Approval at start: LRN 100000000004-015. Incomplete (no TLE grade): LRN 100000000099 and 100000000100. No Approved records at start.</t>
         </is>
       </c>
     </row>
@@ -978,7 +978,7 @@
       </c>
       <c r="B39" s="24" t="inlineStr">
         <is>
-          <t>LRN 100000000001 (Adrian Aguilar). Sample Grade 4 and 5 history; readiness PARTIAL.</t>
+          <t>LRN 100000000001 (Adrian Aguilar). Sample Grade 4 and 5 history; readiness PARTIAL. Grade 6 prints as Terms 1-3 only after approval (D-05).</t>
         </is>
       </c>
     </row>
@@ -4120,12 +4120,12 @@
       </c>
       <c r="I48" s="13" t="inlineStr">
         <is>
-          <t>1. Try to download the SF10 of any other Rizal learner.</t>
+          <t>1. Try to download the SF10 of a Rizal learner who is not approved.</t>
         </is>
       </c>
       <c r="J48" s="13" t="inlineStr">
         <is>
-          <t>e.g. LRN 100000000004</t>
+          <t>e.g. LRN 100000000020 (never submitted or approved in the session)</t>
         </is>
       </c>
       <c r="K48" s="13" t="inlineStr">
@@ -5730,7 +5730,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="19" t="inlineStr">
         <is>
@@ -5826,8 +5825,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="19" t="inlineStr">
         <is>
@@ -6554,8 +6551,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Handoff v15; update D-04 and TC-041 for the per-learner upload lock
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03-Testing/EduCheck_UAT_Test_Cases.xlsx
+++ b/03-Testing/EduCheck_UAT_Test_Cases.xlsx
@@ -3727,7 +3727,7 @@
       </c>
       <c r="G42" s="13" t="inlineStr">
         <is>
-          <t>Approved record is locked against re-upload</t>
+          <t>Approved learner is locked against re-upload</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="K42" s="13" t="inlineStr">
         <is>
-          <t>The upload is refused because the record is approved.</t>
+          <t>The upload is accepted for the rest of the class. The result page lists the approved learner as not updated, and that learner's grades and Approved status do not change.</t>
         </is>
       </c>
       <c r="L42" s="16" t="n"/>

</xml_diff>

<commit_message>
Record the manual test case results and add them to the black-box report
TC-052 to TC-060 and TC-063 to TC-066 passed when run by hand at the
2026-10-16 UAT. The report now reads them from the UAT workbook and shows
76 of 76 passed (63 automated, 13 manual).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03-Testing/EduCheck_UAT_Test_Cases.xlsx
+++ b/03-Testing/EduCheck_UAT_Test_Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/998bf0dccc2814d1/Documents/GitHub/Capstone-Project_EduCheck/03-Testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_C1F5BA203F8BA9F4AE009BB4139EBEDC2939DAAE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="11_C1F5BA203F8BA9F4AE009BB4139EBEDC2939DAAE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF5645EF-A61C-4190-AC0B-0DB59C8CD1E5}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="11712" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="667">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="667">
   <si>
     <t>EduCheck - User Acceptance Test Cases</t>
   </si>
@@ -5165,9 +5165,15 @@
         <v>409</v>
       </c>
       <c r="L53" s="16"/>
-      <c r="M53" s="17"/>
-      <c r="N53" s="16"/>
-      <c r="O53" s="18"/>
+      <c r="M53" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N53" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O53" s="18">
+        <v>46311</v>
+      </c>
       <c r="P53" s="17"/>
       <c r="Q53" s="16"/>
     </row>
@@ -5206,9 +5212,15 @@
         <v>414</v>
       </c>
       <c r="L54" s="16"/>
-      <c r="M54" s="17"/>
-      <c r="N54" s="16"/>
-      <c r="O54" s="18"/>
+      <c r="M54" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N54" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O54" s="18">
+        <v>46311</v>
+      </c>
       <c r="P54" s="17"/>
       <c r="Q54" s="16"/>
     </row>
@@ -5247,9 +5259,15 @@
         <v>419</v>
       </c>
       <c r="L55" s="16"/>
-      <c r="M55" s="17"/>
-      <c r="N55" s="16"/>
-      <c r="O55" s="18"/>
+      <c r="M55" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N55" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O55" s="18">
+        <v>46311</v>
+      </c>
       <c r="P55" s="17"/>
       <c r="Q55" s="16"/>
     </row>
@@ -5288,9 +5306,15 @@
         <v>423</v>
       </c>
       <c r="L56" s="16"/>
-      <c r="M56" s="17"/>
-      <c r="N56" s="16"/>
-      <c r="O56" s="18"/>
+      <c r="M56" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N56" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O56" s="18">
+        <v>46311</v>
+      </c>
       <c r="P56" s="17"/>
       <c r="Q56" s="16"/>
     </row>
@@ -5329,9 +5353,15 @@
         <v>428</v>
       </c>
       <c r="L57" s="16"/>
-      <c r="M57" s="17"/>
-      <c r="N57" s="16"/>
-      <c r="O57" s="18"/>
+      <c r="M57" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N57" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O57" s="18">
+        <v>46311</v>
+      </c>
       <c r="P57" s="17"/>
       <c r="Q57" s="16"/>
     </row>
@@ -5370,9 +5400,15 @@
         <v>432</v>
       </c>
       <c r="L58" s="16"/>
-      <c r="M58" s="17"/>
-      <c r="N58" s="16"/>
-      <c r="O58" s="18"/>
+      <c r="M58" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N58" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O58" s="18">
+        <v>46311</v>
+      </c>
       <c r="P58" s="17"/>
       <c r="Q58" s="16"/>
     </row>
@@ -5411,9 +5447,15 @@
         <v>438</v>
       </c>
       <c r="L59" s="16"/>
-      <c r="M59" s="17"/>
-      <c r="N59" s="16"/>
-      <c r="O59" s="18"/>
+      <c r="M59" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N59" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O59" s="18">
+        <v>46311</v>
+      </c>
       <c r="P59" s="17"/>
       <c r="Q59" s="16"/>
     </row>
@@ -5452,9 +5494,15 @@
         <v>444</v>
       </c>
       <c r="L60" s="16"/>
-      <c r="M60" s="17"/>
-      <c r="N60" s="16"/>
-      <c r="O60" s="18"/>
+      <c r="M60" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N60" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O60" s="18">
+        <v>46311</v>
+      </c>
       <c r="P60" s="17"/>
       <c r="Q60" s="16"/>
     </row>
@@ -5493,9 +5541,15 @@
         <v>449</v>
       </c>
       <c r="L61" s="16"/>
-      <c r="M61" s="17"/>
-      <c r="N61" s="16"/>
-      <c r="O61" s="18"/>
+      <c r="M61" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N61" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O61" s="18">
+        <v>46311</v>
+      </c>
       <c r="P61" s="17"/>
       <c r="Q61" s="16"/>
     </row>
@@ -5616,9 +5670,15 @@
         <v>465</v>
       </c>
       <c r="L64" s="16"/>
-      <c r="M64" s="17"/>
-      <c r="N64" s="16"/>
-      <c r="O64" s="18"/>
+      <c r="M64" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N64" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O64" s="18">
+        <v>46311</v>
+      </c>
       <c r="P64" s="17"/>
       <c r="Q64" s="16"/>
     </row>
@@ -5657,9 +5717,15 @@
         <v>470</v>
       </c>
       <c r="L65" s="16"/>
-      <c r="M65" s="17"/>
-      <c r="N65" s="16"/>
-      <c r="O65" s="18"/>
+      <c r="M65" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N65" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O65" s="18">
+        <v>46311</v>
+      </c>
       <c r="P65" s="17"/>
       <c r="Q65" s="16"/>
     </row>
@@ -5698,9 +5764,15 @@
         <v>475</v>
       </c>
       <c r="L66" s="16"/>
-      <c r="M66" s="17"/>
-      <c r="N66" s="16"/>
-      <c r="O66" s="18"/>
+      <c r="M66" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N66" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O66" s="18">
+        <v>46311</v>
+      </c>
       <c r="P66" s="17"/>
       <c r="Q66" s="16"/>
     </row>
@@ -5739,9 +5811,15 @@
         <v>480</v>
       </c>
       <c r="L67" s="16"/>
-      <c r="M67" s="17"/>
-      <c r="N67" s="16"/>
-      <c r="O67" s="18"/>
+      <c r="M67" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="N67" s="16" t="s">
+        <v>573</v>
+      </c>
+      <c r="O67" s="18">
+        <v>46311</v>
+      </c>
       <c r="P67" s="17"/>
       <c r="Q67" s="16"/>
     </row>
@@ -6223,7 +6301,7 @@
       </c>
       <c r="B6" s="20">
         <f>COUNTIF('Test Cases'!$M$2:$M$77,"Pass")</f>
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
@@ -6250,7 +6328,7 @@
       </c>
       <c r="B9" s="20">
         <f>B5-B6-B7-B8</f>
-        <v>76</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -6259,16 +6337,16 @@
       </c>
       <c r="B10" s="20">
         <f>B6+B7</f>
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>550</v>
       </c>
-      <c r="B11" s="21" t="str">
+      <c r="B11" s="21">
         <f>IF(B10=0,"-",B6/B10)</f>
-        <v>-</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -6277,7 +6355,7 @@
       </c>
       <c r="B12" s="21">
         <f>IF(B5=0,"-",(B10+B8)/B5)</f>
-        <v>0</v>
+        <v>0.17105263157894737</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -6811,7 +6889,7 @@
       </c>
       <c r="C34" s="20">
         <f>COUNTIFS('Test Cases'!$B$2:$B$77,A34,'Test Cases'!$M$2:$M$77,"Pass")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D34" s="20">
         <f>COUNTIFS('Test Cases'!$B$2:$B$77,A34,'Test Cases'!$M$2:$M$77,"Fail")</f>
@@ -6823,11 +6901,11 @@
       </c>
       <c r="F34" s="20">
         <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-      <c r="G34" s="21" t="str">
+        <v>0</v>
+      </c>
+      <c r="G34" s="21">
         <f t="shared" si="1"/>
-        <v>-</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
@@ -6869,7 +6947,7 @@
       </c>
       <c r="C36" s="20">
         <f>COUNTIFS('Test Cases'!$B$2:$B$77,A36,'Test Cases'!$M$2:$M$77,"Pass")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D36" s="20">
         <f>COUNTIFS('Test Cases'!$B$2:$B$77,A36,'Test Cases'!$M$2:$M$77,"Fail")</f>
@@ -6881,11 +6959,11 @@
       </c>
       <c r="F36" s="20">
         <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="G36" s="21" t="str">
+        <v>0</v>
+      </c>
+      <c r="G36" s="21">
         <f t="shared" si="1"/>
-        <v>-</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
@@ -6898,7 +6976,7 @@
       </c>
       <c r="C37" s="20">
         <f>COUNTIFS('Test Cases'!$B$2:$B$77,A37,'Test Cases'!$M$2:$M$77,"Pass")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D37" s="20">
         <f>COUNTIFS('Test Cases'!$B$2:$B$77,A37,'Test Cases'!$M$2:$M$77,"Fail")</f>
@@ -6910,11 +6988,11 @@
       </c>
       <c r="F37" s="20">
         <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="G37" s="21" t="str">
+        <v>0</v>
+      </c>
+      <c r="G37" s="21">
         <f t="shared" si="1"/>
-        <v>-</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
@@ -6984,7 +7062,7 @@
       </c>
       <c r="C43" s="20">
         <f>COUNTIFS('Test Cases'!$E$2:$E$77,A43,'Test Cases'!$M$2:$M$77,"Pass")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D43" s="20">
         <f>COUNTIFS('Test Cases'!$E$2:$E$77,A43,'Test Cases'!$M$2:$M$77,"Fail")</f>
@@ -6996,11 +7074,11 @@
       </c>
       <c r="F43" s="20">
         <f t="shared" ref="F43:F48" si="2">B43-C43-D43-E43</f>
-        <v>19</v>
-      </c>
-      <c r="G43" s="21" t="str">
+        <v>17</v>
+      </c>
+      <c r="G43" s="21">
         <f t="shared" ref="G43:G48" si="3">IF(C43+D43=0,"-",C43/(C43+D43))</f>
-        <v>-</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
@@ -7013,7 +7091,7 @@
       </c>
       <c r="C44" s="20">
         <f>COUNTIFS('Test Cases'!$E$2:$E$77,A44,'Test Cases'!$M$2:$M$77,"Pass")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D44" s="20">
         <f>COUNTIFS('Test Cases'!$E$2:$E$77,A44,'Test Cases'!$M$2:$M$77,"Fail")</f>
@@ -7025,11 +7103,11 @@
       </c>
       <c r="F44" s="20">
         <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="G44" s="21" t="str">
+        <v>2</v>
+      </c>
+      <c r="G44" s="21">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
@@ -7042,7 +7120,7 @@
       </c>
       <c r="C45" s="20">
         <f>COUNTIFS('Test Cases'!$E$2:$E$77,A45,'Test Cases'!$M$2:$M$77,"Pass")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D45" s="20">
         <f>COUNTIFS('Test Cases'!$E$2:$E$77,A45,'Test Cases'!$M$2:$M$77,"Fail")</f>
@@ -7054,11 +7132,11 @@
       </c>
       <c r="F45" s="20">
         <f t="shared" si="2"/>
-        <v>47</v>
-      </c>
-      <c r="G45" s="21" t="str">
+        <v>42</v>
+      </c>
+      <c r="G45" s="21">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
@@ -7071,7 +7149,7 @@
       </c>
       <c r="C46" s="20">
         <f>COUNTIFS('Test Cases'!$E$2:$E$77,A46,'Test Cases'!$M$2:$M$77,"Pass")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D46" s="20">
         <f>COUNTIFS('Test Cases'!$E$2:$E$77,A46,'Test Cases'!$M$2:$M$77,"Fail")</f>
@@ -7083,11 +7161,11 @@
       </c>
       <c r="F46" s="20">
         <f t="shared" si="2"/>
-        <v>3</v>
-      </c>
-      <c r="G46" s="21" t="str">
+        <v>0</v>
+      </c>
+      <c r="G46" s="21">
         <f t="shared" si="3"/>
-        <v>-</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
@@ -7100,7 +7178,7 @@
       </c>
       <c r="C47" s="20">
         <f>COUNTIFS('Test Cases'!$E$2:$E$77,A47,'Test Cases'!$M$2:$M$77,"Pass")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D47" s="20">
         <f>COUNTIFS('Test Cases'!$E$2:$E$77,A47,'Test Cases'!$M$2:$M$77,"Fail")</f>
@@ -7112,11 +7190,11 @@
       </c>
       <c r="F47" s="20">
         <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G47" s="21">
+        <f t="shared" si="3"/>
         <v>1</v>
-      </c>
-      <c r="G47" s="21" t="str">
-        <f t="shared" si="3"/>
-        <v>-</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Add the evaluation results and a Results and Discussion draft
The ISO/IEC 25010, SUS and heuristic responses from the online testing at
Atimonan Central School Annex and East 8 Elementary School are tabulated:
ISO overall 4.38 (school personnel) and 4.85 (IT expert), SUS 66.0, heuristic
mean severity 0.15. The draft covers Objectives 4 and 5 and discusses the
lowest scores. The manual test cases are dated 2026-10-15 (Atimonan).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03-Testing/EduCheck_UAT_Test_Cases.xlsx
+++ b/03-Testing/EduCheck_UAT_Test_Cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/998bf0dccc2814d1/Documents/GitHub/Capstone-Project_EduCheck/03-Testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="11_C1F5BA203F8BA9F4AE009BB4139EBEDC2939DAAE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF5645EF-A61C-4190-AC0B-0DB59C8CD1E5}"/>
+  <xr:revisionPtr revIDLastSave="78" documentId="11_C1F5BA203F8BA9F4AE009BB4139EBEDC2939DAAE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C5A46DE-A9AB-46F7-A2A5-2FB0AD72CC6E}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11712" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -2334,6 +2334,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5172,7 +5176,7 @@
         <v>573</v>
       </c>
       <c r="O53" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P53" s="17"/>
       <c r="Q53" s="16"/>
@@ -5219,7 +5223,7 @@
         <v>573</v>
       </c>
       <c r="O54" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P54" s="17"/>
       <c r="Q54" s="16"/>
@@ -5266,7 +5270,7 @@
         <v>573</v>
       </c>
       <c r="O55" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P55" s="17"/>
       <c r="Q55" s="16"/>
@@ -5313,7 +5317,7 @@
         <v>573</v>
       </c>
       <c r="O56" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P56" s="17"/>
       <c r="Q56" s="16"/>
@@ -5360,7 +5364,7 @@
         <v>573</v>
       </c>
       <c r="O57" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P57" s="17"/>
       <c r="Q57" s="16"/>
@@ -5407,7 +5411,7 @@
         <v>573</v>
       </c>
       <c r="O58" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P58" s="17"/>
       <c r="Q58" s="16"/>
@@ -5454,7 +5458,7 @@
         <v>573</v>
       </c>
       <c r="O59" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P59" s="17"/>
       <c r="Q59" s="16"/>
@@ -5501,7 +5505,7 @@
         <v>573</v>
       </c>
       <c r="O60" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P60" s="17"/>
       <c r="Q60" s="16"/>
@@ -5548,7 +5552,7 @@
         <v>573</v>
       </c>
       <c r="O61" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P61" s="17"/>
       <c r="Q61" s="16"/>
@@ -5677,7 +5681,7 @@
         <v>573</v>
       </c>
       <c r="O64" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P64" s="17"/>
       <c r="Q64" s="16"/>
@@ -5724,7 +5728,7 @@
         <v>573</v>
       </c>
       <c r="O65" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P65" s="17"/>
       <c r="Q65" s="16"/>
@@ -5771,7 +5775,7 @@
         <v>573</v>
       </c>
       <c r="O66" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P66" s="17"/>
       <c r="Q66" s="16"/>
@@ -5818,7 +5822,7 @@
         <v>573</v>
       </c>
       <c r="O67" s="18">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="P67" s="17"/>
       <c r="Q67" s="16"/>

</xml_diff>

<commit_message>
Mark TC-002, TC-051 and TC-062 as passed with remarks
The automated report gets a "Pass with remarks" result (60 pass, 3 with
remarks, 13 manual pass), and the UAT workbook's Remarks column explains
each one, matching the Results and Discussion draft.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03-Testing/EduCheck_UAT_Test_Cases.xlsx
+++ b/03-Testing/EduCheck_UAT_Test_Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/998bf0dccc2814d1/Documents/GitHub/Capstone-Project_EduCheck/03-Testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="78" documentId="11_C1F5BA203F8BA9F4AE009BB4139EBEDC2939DAAE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C5A46DE-A9AB-46F7-A2A5-2FB0AD72CC6E}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="11_C1F5BA203F8BA9F4AE009BB4139EBEDC2939DAAE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68F26646-EBB3-4A0C-9456-35907B022EF1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="667">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="670">
   <si>
     <t>EduCheck - User Acceptance Test Cases</t>
   </si>
@@ -2125,6 +2125,15 @@
   </si>
   <si>
     <t>Cosmetic: layout, wording, alignment.</t>
+  </si>
+  <si>
+    <t>Automated run 2026-10-23: Pass with remarks. The message reads "Username or password is incorrect. Check both and try again." instead of "Invalid username or password."; it still does not say which field was wrong.</t>
+  </si>
+  <si>
+    <t>Automated run 2026-10-23: Pass with remarks. The unread count on the Notifications page drops to 0 at once; the sidebar badge updates only after the page is refreshed.</t>
+  </si>
+  <si>
+    <t>Automated run 2026-10-23: Pass with remarks. Measured on the local server only; the first load of the hosted (Render) system is still slow (DEF-003).</t>
   </si>
 </sst>
 </file>
@@ -3123,7 +3132,9 @@
       <c r="N3" s="16"/>
       <c r="O3" s="18"/>
       <c r="P3" s="17"/>
-      <c r="Q3" s="16"/>
+      <c r="Q3" s="16" t="s">
+        <v>667</v>
+      </c>
     </row>
     <row r="4" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
@@ -5132,7 +5143,9 @@
       <c r="N52" s="16"/>
       <c r="O52" s="18"/>
       <c r="P52" s="17"/>
-      <c r="Q52" s="16"/>
+      <c r="Q52" s="16" t="s">
+        <v>668</v>
+      </c>
     </row>
     <row r="53" spans="1:17" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="14" t="s">
@@ -5637,7 +5650,9 @@
       <c r="N63" s="16"/>
       <c r="O63" s="18"/>
       <c r="P63" s="17"/>
-      <c r="Q63" s="16"/>
+      <c r="Q63" s="16" t="s">
+        <v>669</v>
+      </c>
     </row>
     <row r="64" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="14" t="s">

</xml_diff>